<commit_message>
Updated outputs and project structure file
</commit_message>
<xml_diff>
--- a/CAD/Outputs/BOM/Bill of Materials-BioZSpec.xlsx
+++ b/CAD/Outputs/BOM/Bill of Materials-BioZSpec.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sunray\Documents\Bioimpedance AFE\CAD\Outputs\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF600AF4-E2BB-4111-95B0-2CA49B2706C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E6C9B5B-BAE4-442E-8A3C-156B6EB3E722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3525" yWindow="3435" windowWidth="21600" windowHeight="11385" xr2:uid="{10FF59C9-E279-43AF-988B-0CF057D2FF91}"/>
+    <workbookView xWindow="3525" yWindow="3435" windowWidth="21600" windowHeight="11385" xr2:uid="{9CF62104-0C2D-4A2A-943D-F305011BD6E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-BioZSpec" sheetId="1" r:id="rId1"/>
@@ -1139,7 +1139,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F41A2FE-2118-4E69-8BAC-C9C9E1AA8017}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A768412-7ECE-4102-8DD4-89A4870CB69A}">
   <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
Re-added ground stitch pattern
</commit_message>
<xml_diff>
--- a/CAD/Outputs/BOM/Bill of Materials-BioZSpec.xlsx
+++ b/CAD/Outputs/BOM/Bill of Materials-BioZSpec.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sunray\Documents\Bioimpedance AFE\CAD\Outputs\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E6C9B5B-BAE4-442E-8A3C-156B6EB3E722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE51ED28-40EB-4907-8C56-D288A22FE6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3525" yWindow="3435" windowWidth="21600" windowHeight="11385" xr2:uid="{9CF62104-0C2D-4A2A-943D-F305011BD6E1}"/>
+    <workbookView xWindow="3525" yWindow="3435" windowWidth="21600" windowHeight="11385" xr2:uid="{5F672218-90AB-4E5C-A118-3EA2F487EDE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-BioZSpec" sheetId="1" r:id="rId1"/>
@@ -1139,7 +1139,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A768412-7ECE-4102-8DD4-89A4870CB69A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ADF1E6C-FFA8-4673-95F6-6DE0BD07D76A}">
   <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>